<commit_message>
se hiso la limpieza de los datos que contenia las tabla de promedio de uso de celular al dia
</commit_message>
<xml_diff>
--- a/Short_Laprida_Sian_TPINTEGRADOR.xlsx
+++ b/Short_Laprida_Sian_TPINTEGRADOR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\short\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IPF-2026\Desktop\trabajos\Matematica\Estadistica-Trabajo-integrador-Short-Laprida-Sian\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F094D2DC-45AB-4F61-B283-C55D445FDD4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B79EB78-24DC-41FA-8B92-7F37DAA2D47D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{98BD9788-430D-4B00-92BA-E7D9A5175AA6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{98BD9788-430D-4B00-92BA-E7D9A5175AA6}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -801,17 +801,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32094DED-D156-4F92-A985-06D8DE97CBA2}">
   <dimension ref="C2:L213"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="6" max="6" width="18.28515625" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" customWidth="1"/>
+    <col min="6" max="6" width="18.33203125" customWidth="1"/>
+    <col min="7" max="7" width="14.88671875" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="22" customWidth="1"/>
-    <col min="10" max="11" width="16.140625" customWidth="1"/>
+    <col min="10" max="11" width="16.109375" customWidth="1"/>
     <col min="12" max="12" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="3:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -843,7 +843,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C3" s="1" t="s">
         <v>10</v>
       </c>
@@ -875,7 +875,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C4" s="1" t="s">
         <v>11</v>
       </c>
@@ -907,7 +907,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C5" s="1" t="s">
         <v>11</v>
       </c>
@@ -939,7 +939,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C6" s="1" t="s">
         <v>10</v>
       </c>
@@ -971,7 +971,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C7" s="1" t="s">
         <v>10</v>
       </c>
@@ -1003,7 +1003,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C8" s="1" t="s">
         <v>11</v>
       </c>
@@ -1035,7 +1035,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C9" s="1" t="s">
         <v>12</v>
       </c>
@@ -1067,7 +1067,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C10" s="1" t="s">
         <v>11</v>
       </c>
@@ -1099,7 +1099,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C11" s="1" t="s">
         <v>10</v>
       </c>
@@ -1131,7 +1131,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C12" s="1" t="s">
         <v>10</v>
       </c>
@@ -1163,7 +1163,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C13" s="1" t="s">
         <v>11</v>
       </c>
@@ -1195,7 +1195,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C14" s="1" t="s">
         <v>11</v>
       </c>
@@ -1227,7 +1227,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C15" s="1" t="s">
         <v>10</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C16" s="1" t="s">
         <v>10</v>
       </c>
@@ -1291,7 +1291,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C17" s="1" t="s">
         <v>11</v>
       </c>
@@ -1323,7 +1323,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C18" s="1" t="s">
         <v>10</v>
       </c>
@@ -1355,7 +1355,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C19" s="1" t="s">
         <v>12</v>
       </c>
@@ -1387,7 +1387,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C20" s="1" t="s">
         <v>11</v>
       </c>
@@ -1419,7 +1419,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C21" s="1" t="s">
         <v>10</v>
       </c>
@@ -1451,7 +1451,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C22" s="1" t="s">
         <v>10</v>
       </c>
@@ -1483,7 +1483,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C23" s="1" t="s">
         <v>11</v>
       </c>
@@ -1515,7 +1515,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C24" s="1" t="s">
         <v>11</v>
       </c>
@@ -1547,7 +1547,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1579,7 +1579,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C26" s="1" t="s">
         <v>10</v>
       </c>
@@ -1611,7 +1611,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C27" s="1" t="s">
         <v>11</v>
       </c>
@@ -1643,7 +1643,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C28" s="1" t="s">
         <v>12</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C29" s="1" t="s">
         <v>11</v>
       </c>
@@ -1707,7 +1707,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C30" s="1" t="s">
         <v>10</v>
       </c>
@@ -1739,7 +1739,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C31" s="1" t="s">
         <v>10</v>
       </c>
@@ -1771,7 +1771,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C32" s="1" t="s">
         <v>11</v>
       </c>
@@ -1803,7 +1803,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C33" s="1" t="s">
         <v>11</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C34" s="1" t="s">
         <v>10</v>
       </c>
@@ -1867,7 +1867,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C35" s="1" t="s">
         <v>10</v>
       </c>
@@ -1899,7 +1899,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C36" s="1" t="s">
         <v>11</v>
       </c>
@@ -1931,7 +1931,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C37" s="1" t="s">
         <v>10</v>
       </c>
@@ -1963,7 +1963,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C38" s="1" t="s">
         <v>12</v>
       </c>
@@ -1995,7 +1995,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C39" s="1" t="s">
         <v>11</v>
       </c>
@@ -2027,7 +2027,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="40" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C40" s="1" t="s">
         <v>10</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C41" s="1" t="s">
         <v>10</v>
       </c>
@@ -2091,7 +2091,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C42" s="1" t="s">
         <v>11</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C43" s="1" t="s">
         <v>11</v>
       </c>
@@ -2155,7 +2155,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C44" s="1" t="s">
         <v>10</v>
       </c>
@@ -2187,7 +2187,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C45" s="1" t="s">
         <v>10</v>
       </c>
@@ -2219,7 +2219,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C46" s="1" t="s">
         <v>11</v>
       </c>
@@ -2251,7 +2251,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C47" s="1" t="s">
         <v>12</v>
       </c>
@@ -2283,7 +2283,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C48" s="1" t="s">
         <v>11</v>
       </c>
@@ -2315,7 +2315,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C49" s="1" t="s">
         <v>10</v>
       </c>
@@ -2347,7 +2347,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C50" s="1" t="s">
         <v>10</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="51" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C51" s="1" t="s">
         <v>11</v>
       </c>
@@ -2411,7 +2411,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C52" s="1" t="s">
         <v>11</v>
       </c>
@@ -2443,7 +2443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="53" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C53" s="1" t="s">
         <v>10</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="54" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C54" s="1" t="s">
         <v>10</v>
       </c>
@@ -2507,7 +2507,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="55" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C55" s="1" t="s">
         <v>11</v>
       </c>
@@ -2539,7 +2539,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="56" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="56" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C56" s="1" t="s">
         <v>10</v>
       </c>
@@ -2571,7 +2571,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="57" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="57" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C57" s="1" t="s">
         <v>12</v>
       </c>
@@ -2603,7 +2603,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="58" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="58" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C58" s="1" t="s">
         <v>11</v>
       </c>
@@ -2635,7 +2635,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="59" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C59" s="1" t="s">
         <v>10</v>
       </c>
@@ -2667,7 +2667,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="60" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C60" s="1" t="s">
         <v>10</v>
       </c>
@@ -2699,7 +2699,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="61" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C61" s="1" t="s">
         <v>11</v>
       </c>
@@ -2731,7 +2731,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="62" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C62" s="1" t="s">
         <v>11</v>
       </c>
@@ -2763,7 +2763,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="63" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="63" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C63" s="1" t="s">
         <v>10</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="64" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C64" s="1" t="s">
         <v>10</v>
       </c>
@@ -2827,7 +2827,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="65" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="65" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C65" s="1" t="s">
         <v>11</v>
       </c>
@@ -2859,7 +2859,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="66" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C66" s="1" t="s">
         <v>12</v>
       </c>
@@ -2891,7 +2891,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="67" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C67" s="1" t="s">
         <v>11</v>
       </c>
@@ -2923,7 +2923,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="68" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C68" s="1" t="s">
         <v>10</v>
       </c>
@@ -2955,7 +2955,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="69" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="69" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C69" s="1" t="s">
         <v>10</v>
       </c>
@@ -2987,7 +2987,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="70" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="70" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C70" s="1" t="s">
         <v>11</v>
       </c>
@@ -3019,7 +3019,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="71" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="71" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C71" s="1" t="s">
         <v>11</v>
       </c>
@@ -3051,7 +3051,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="72" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C72" s="1" t="s">
         <v>10</v>
       </c>
@@ -3083,7 +3083,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="73" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="73" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C73" s="1" t="s">
         <v>10</v>
       </c>
@@ -3115,7 +3115,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="74" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="74" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C74" s="1" t="s">
         <v>11</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="75" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C75" s="1" t="s">
         <v>10</v>
       </c>
@@ -3179,7 +3179,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="76" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="76" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C76" s="1" t="s">
         <v>12</v>
       </c>
@@ -3211,7 +3211,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="77" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="77" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C77" s="1" t="s">
         <v>11</v>
       </c>
@@ -3243,7 +3243,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="78" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="78" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C78" s="1" t="s">
         <v>10</v>
       </c>
@@ -3275,7 +3275,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="79" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="79" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C79" s="1" t="s">
         <v>10</v>
       </c>
@@ -3307,7 +3307,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="80" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="80" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C80" s="1" t="s">
         <v>11</v>
       </c>
@@ -3339,7 +3339,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="81" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="81" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C81" s="1" t="s">
         <v>11</v>
       </c>
@@ -3371,7 +3371,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="82" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="82" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C82" s="1" t="s">
         <v>10</v>
       </c>
@@ -3403,7 +3403,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="83" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="83" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C83" s="1" t="s">
         <v>10</v>
       </c>
@@ -3435,7 +3435,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="84" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="84" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C84" s="1" t="s">
         <v>11</v>
       </c>
@@ -3467,7 +3467,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="85" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="85" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C85" s="1" t="s">
         <v>12</v>
       </c>
@@ -3499,7 +3499,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="86" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="86" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C86" s="1" t="s">
         <v>11</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="87" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="87" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C87" s="1" t="s">
         <v>10</v>
       </c>
@@ -3563,7 +3563,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="88" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="88" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C88" s="1" t="s">
         <v>10</v>
       </c>
@@ -3595,7 +3595,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="89" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="89" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C89" s="1" t="s">
         <v>11</v>
       </c>
@@ -3627,7 +3627,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="90" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="90" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C90" s="1" t="s">
         <v>11</v>
       </c>
@@ -3659,7 +3659,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="91" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="91" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C91" s="1" t="s">
         <v>10</v>
       </c>
@@ -3691,7 +3691,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="92" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="92" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C92" s="1" t="s">
         <v>10</v>
       </c>
@@ -3723,7 +3723,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="93" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="93" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C93" s="1" t="s">
         <v>11</v>
       </c>
@@ -3755,7 +3755,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="94" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="94" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C94" s="1" t="s">
         <v>10</v>
       </c>
@@ -3787,7 +3787,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="95" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="95" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C95" s="1" t="s">
         <v>12</v>
       </c>
@@ -3819,7 +3819,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="96" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="96" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C96" s="1" t="s">
         <v>11</v>
       </c>
@@ -3851,7 +3851,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="97" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="97" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C97" s="1" t="s">
         <v>10</v>
       </c>
@@ -3883,7 +3883,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="98" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C98" s="1" t="s">
         <v>10</v>
       </c>
@@ -3915,7 +3915,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="99" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="99" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C99" s="1" t="s">
         <v>11</v>
       </c>
@@ -3947,7 +3947,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="100" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="100" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C100" s="1" t="s">
         <v>11</v>
       </c>
@@ -3979,7 +3979,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="101" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="101" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C101" s="1" t="s">
         <v>10</v>
       </c>
@@ -4011,7 +4011,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="102" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="102" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C102" s="1" t="s">
         <v>10</v>
       </c>
@@ -4043,7 +4043,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="103" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="103" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C103" s="1" t="s">
         <v>11</v>
       </c>
@@ -4075,7 +4075,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="104" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C104" s="1" t="s">
         <v>12</v>
       </c>
@@ -4107,7 +4107,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="105" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="105" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C105" s="1" t="s">
         <v>11</v>
       </c>
@@ -4139,7 +4139,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="106" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="106" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C106" s="1" t="s">
         <v>10</v>
       </c>
@@ -4171,7 +4171,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="107" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="107" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C107" s="1" t="s">
         <v>10</v>
       </c>
@@ -4203,7 +4203,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="108" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="108" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C108" s="1" t="s">
         <v>11</v>
       </c>
@@ -4235,7 +4235,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="109" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="109" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C109" s="1" t="s">
         <v>11</v>
       </c>
@@ -4267,7 +4267,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="110" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="110" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C110" s="1" t="s">
         <v>10</v>
       </c>
@@ -4299,7 +4299,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="111" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="111" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C111" s="1" t="s">
         <v>10</v>
       </c>
@@ -4331,7 +4331,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="112" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="112" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C112" s="1" t="s">
         <v>11</v>
       </c>
@@ -4363,7 +4363,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="113" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="113" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C113" s="1" t="s">
         <v>10</v>
       </c>
@@ -4395,7 +4395,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="114" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="114" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C114" s="1" t="s">
         <v>12</v>
       </c>
@@ -4427,7 +4427,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="115" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="115" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C115" s="1" t="s">
         <v>11</v>
       </c>
@@ -4459,7 +4459,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="116" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="116" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C116" s="1" t="s">
         <v>10</v>
       </c>
@@ -4491,7 +4491,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="117" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C117" s="1" t="s">
         <v>10</v>
       </c>
@@ -4523,7 +4523,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="118" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="118" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C118" s="1" t="s">
         <v>11</v>
       </c>
@@ -4555,7 +4555,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="119" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="119" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C119" s="1" t="s">
         <v>11</v>
       </c>
@@ -4587,7 +4587,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="120" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="120" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C120" s="1" t="s">
         <v>10</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="121" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="121" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C121" s="1" t="s">
         <v>10</v>
       </c>
@@ -4651,7 +4651,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="122" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="122" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C122" s="1" t="s">
         <v>11</v>
       </c>
@@ -4683,7 +4683,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="123" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="123" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C123" s="1" t="s">
         <v>12</v>
       </c>
@@ -4715,7 +4715,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="124" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="124" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C124" s="1" t="s">
         <v>11</v>
       </c>
@@ -4747,7 +4747,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="125" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="125" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C125" s="1" t="s">
         <v>10</v>
       </c>
@@ -4779,7 +4779,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="126" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="126" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C126" s="1" t="s">
         <v>10</v>
       </c>
@@ -4811,7 +4811,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="127" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="127" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C127" s="1" t="s">
         <v>11</v>
       </c>
@@ -4843,7 +4843,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="128" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="128" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C128" s="1" t="s">
         <v>11</v>
       </c>
@@ -4875,7 +4875,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="129" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="129" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C129" s="1" t="s">
         <v>10</v>
       </c>
@@ -4907,7 +4907,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="130" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="130" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C130" s="1" t="s">
         <v>10</v>
       </c>
@@ -4939,7 +4939,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="131" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="131" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C131" s="1" t="s">
         <v>11</v>
       </c>
@@ -4971,7 +4971,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="132" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="132" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C132" s="1" t="s">
         <v>10</v>
       </c>
@@ -5003,7 +5003,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="133" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="133" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C133" s="1" t="s">
         <v>12</v>
       </c>
@@ -5035,7 +5035,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="134" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="134" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C134" s="1" t="s">
         <v>11</v>
       </c>
@@ -5067,7 +5067,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="135" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="135" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C135" s="1" t="s">
         <v>10</v>
       </c>
@@ -5099,7 +5099,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="136" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="136" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C136" s="1" t="s">
         <v>10</v>
       </c>
@@ -5131,7 +5131,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="137" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="137" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C137" s="1" t="s">
         <v>11</v>
       </c>
@@ -5163,7 +5163,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="138" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="138" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C138" s="1" t="s">
         <v>11</v>
       </c>
@@ -5195,7 +5195,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="139" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="139" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C139" s="1" t="s">
         <v>10</v>
       </c>
@@ -5227,7 +5227,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="140" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="140" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C140" s="1" t="s">
         <v>10</v>
       </c>
@@ -5259,7 +5259,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="141" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="141" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C141" s="1" t="s">
         <v>11</v>
       </c>
@@ -5291,7 +5291,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="142" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="142" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C142" s="1" t="s">
         <v>12</v>
       </c>
@@ -5323,7 +5323,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="143" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="143" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C143" s="1" t="s">
         <v>11</v>
       </c>
@@ -5355,7 +5355,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="144" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="144" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C144" s="1" t="s">
         <v>10</v>
       </c>
@@ -5387,7 +5387,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="145" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="145" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C145" s="1" t="s">
         <v>10</v>
       </c>
@@ -5419,7 +5419,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="146" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="146" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C146" s="1" t="s">
         <v>11</v>
       </c>
@@ -5451,7 +5451,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="147" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="147" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C147" s="1" t="s">
         <v>11</v>
       </c>
@@ -5483,7 +5483,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="148" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="148" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C148" s="1" t="s">
         <v>10</v>
       </c>
@@ -5515,7 +5515,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="149" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="149" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C149" s="1" t="s">
         <v>10</v>
       </c>
@@ -5547,7 +5547,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="150" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="150" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C150" s="1" t="s">
         <v>11</v>
       </c>
@@ -5579,7 +5579,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="151" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="151" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C151" s="1" t="s">
         <v>10</v>
       </c>
@@ -5611,7 +5611,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="152" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="152" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C152" s="1" t="s">
         <v>12</v>
       </c>
@@ -5643,7 +5643,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="153" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="153" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C153" s="1" t="s">
         <v>11</v>
       </c>
@@ -5675,7 +5675,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="154" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="154" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C154" s="1" t="s">
         <v>10</v>
       </c>
@@ -5707,7 +5707,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="155" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="155" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C155" s="1" t="s">
         <v>10</v>
       </c>
@@ -5739,7 +5739,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="156" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="156" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C156" s="1" t="s">
         <v>11</v>
       </c>
@@ -5771,7 +5771,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="157" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="157" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C157" s="1" t="s">
         <v>11</v>
       </c>
@@ -5803,7 +5803,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="158" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="158" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C158" s="1" t="s">
         <v>10</v>
       </c>
@@ -5835,7 +5835,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="159" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="159" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C159" s="1" t="s">
         <v>10</v>
       </c>
@@ -5867,7 +5867,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="160" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="160" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C160" s="1" t="s">
         <v>11</v>
       </c>
@@ -5899,7 +5899,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="161" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="161" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C161" s="1" t="s">
         <v>12</v>
       </c>
@@ -5931,7 +5931,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="162" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="162" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C162" s="1" t="s">
         <v>11</v>
       </c>
@@ -5963,7 +5963,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="163" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="163" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C163" s="1" t="s">
         <v>10</v>
       </c>
@@ -5995,7 +5995,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="164" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="164" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C164" s="1" t="s">
         <v>10</v>
       </c>
@@ -6027,7 +6027,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="165" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="165" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C165" s="1" t="s">
         <v>11</v>
       </c>
@@ -6059,7 +6059,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="166" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="166" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C166" s="1" t="s">
         <v>11</v>
       </c>
@@ -6091,7 +6091,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="167" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="167" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C167" s="1" t="s">
         <v>10</v>
       </c>
@@ -6123,7 +6123,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="168" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="168" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C168" s="1" t="s">
         <v>10</v>
       </c>
@@ -6155,7 +6155,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="169" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="169" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C169" s="1" t="s">
         <v>11</v>
       </c>
@@ -6187,7 +6187,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="170" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="170" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C170" s="1" t="s">
         <v>10</v>
       </c>
@@ -6219,7 +6219,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="171" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="171" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C171" s="1" t="s">
         <v>12</v>
       </c>
@@ -6251,7 +6251,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="172" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="172" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C172" s="1" t="s">
         <v>11</v>
       </c>
@@ -6283,7 +6283,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="173" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="173" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C173" s="1" t="s">
         <v>10</v>
       </c>
@@ -6315,7 +6315,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="174" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="174" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C174" s="1" t="s">
         <v>10</v>
       </c>
@@ -6347,7 +6347,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="175" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="175" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C175" s="1" t="s">
         <v>11</v>
       </c>
@@ -6379,7 +6379,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="176" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="176" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C176" s="1" t="s">
         <v>11</v>
       </c>
@@ -6411,7 +6411,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="177" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="177" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C177" s="1" t="s">
         <v>10</v>
       </c>
@@ -6443,7 +6443,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="178" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="178" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C178" s="1" t="s">
         <v>10</v>
       </c>
@@ -6475,7 +6475,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="179" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="179" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C179" s="1" t="s">
         <v>11</v>
       </c>
@@ -6507,7 +6507,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="180" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="180" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C180" s="1" t="s">
         <v>12</v>
       </c>
@@ -6539,7 +6539,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="181" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="181" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C181" s="1" t="s">
         <v>11</v>
       </c>
@@ -6571,7 +6571,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="182" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="182" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C182" s="1" t="s">
         <v>10</v>
       </c>
@@ -6603,7 +6603,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="183" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="183" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C183" s="1" t="s">
         <v>10</v>
       </c>
@@ -6635,7 +6635,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="184" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="184" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C184" s="1" t="s">
         <v>11</v>
       </c>
@@ -6667,7 +6667,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="185" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="185" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C185" s="1" t="s">
         <v>11</v>
       </c>
@@ -6699,7 +6699,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="186" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="186" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C186" s="1" t="s">
         <v>10</v>
       </c>
@@ -6731,7 +6731,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="187" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="187" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C187" s="1" t="s">
         <v>10</v>
       </c>
@@ -6763,7 +6763,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="188" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="188" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C188" s="1" t="s">
         <v>11</v>
       </c>
@@ -6795,7 +6795,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="189" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="189" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C189" s="1" t="s">
         <v>10</v>
       </c>
@@ -6827,7 +6827,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="190" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="190" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C190" s="1" t="s">
         <v>12</v>
       </c>
@@ -6859,7 +6859,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="191" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="191" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C191" s="1" t="s">
         <v>11</v>
       </c>
@@ -6891,7 +6891,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="192" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="192" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C192" s="1" t="s">
         <v>10</v>
       </c>
@@ -6923,7 +6923,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="193" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="193" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C193" s="1" t="s">
         <v>10</v>
       </c>
@@ -6955,7 +6955,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="194" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="194" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C194" s="1" t="s">
         <v>11</v>
       </c>
@@ -6987,7 +6987,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="195" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="195" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C195" s="1" t="s">
         <v>11</v>
       </c>
@@ -7019,7 +7019,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="196" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="196" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C196" s="1" t="s">
         <v>10</v>
       </c>
@@ -7051,7 +7051,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="197" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="197" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C197" s="1" t="s">
         <v>10</v>
       </c>
@@ -7083,7 +7083,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="198" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="198" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C198" s="1" t="s">
         <v>11</v>
       </c>
@@ -7115,7 +7115,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="199" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="199" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C199" s="1" t="s">
         <v>12</v>
       </c>
@@ -7147,7 +7147,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="200" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="200" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C200" s="1" t="s">
         <v>11</v>
       </c>
@@ -7179,7 +7179,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="201" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="201" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C201" s="1" t="s">
         <v>10</v>
       </c>
@@ -7211,7 +7211,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="202" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="202" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C202" s="1" t="s">
         <v>10</v>
       </c>
@@ -7243,7 +7243,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="203" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="203" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C203" s="1" t="s">
         <v>11</v>
       </c>
@@ -7275,7 +7275,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="204" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="204" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C204" s="1" t="s">
         <v>11</v>
       </c>
@@ -7307,7 +7307,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="205" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="205" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C205" s="1" t="s">
         <v>10</v>
       </c>
@@ -7339,7 +7339,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="206" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="206" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C206" s="1" t="s">
         <v>10</v>
       </c>
@@ -7371,7 +7371,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="207" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="207" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C207" s="1" t="s">
         <v>11</v>
       </c>
@@ -7403,7 +7403,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="208" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="208" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C208" s="1" t="s">
         <v>10</v>
       </c>
@@ -7435,7 +7435,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="209" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="209" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C209" s="1" t="s">
         <v>12</v>
       </c>
@@ -7467,7 +7467,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="210" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="210" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C210" s="1" t="s">
         <v>11</v>
       </c>
@@ -7499,7 +7499,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="211" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="211" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C211" s="1" t="s">
         <v>10</v>
       </c>
@@ -7531,7 +7531,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="212" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="212" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C212" s="1" t="s">
         <v>10</v>
       </c>
@@ -7563,7 +7563,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="213" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="213" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C213" s="1" t="s">
         <v>11</v>
       </c>

</xml_diff>